<commit_message>
Source awarded figure to Genus Q4FY26 call (15 crore tendered, May-2026)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Consumer_Metering_Status_Aug2026.xlsx
+++ b/Smart_Consumer_Metering_Status_Aug2026.xlsx
@@ -344,10 +344,10 @@
     <t xml:space="preserve">Nov-24: 16.8 mn (NSGM); Mar-25: 24.0 mn (NSGM via tndindia); mid-25: ~27.7 mn (indiasmartgrid.org); 15-Nov-25: 47.6 mn (Mercom India); 11-Dec-25: 49.3 mn, 1.6 cr prepaid (Power Minister, newsonair.gov.in); 15-Feb-26: 58.3 mn @ ~1.35 lakh/day (PFI/pfie.com); 30-Jun-26: 72.4 mn (Parliament)</t>
   </si>
   <si>
-    <t xml:space="preserve">Awarded ~150 mn (ESTIMATE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No single official 2026 figure. Prayas (Mar-25): ~62% of sanctioned awarded (~138 mn, matches your earlier sheet); Zerodha Daily Brief (mid-25): ~12 crore; further awards through FY26. 150 mn is an estimate — flagged yellow.</t>
+    <t xml:space="preserve">Awarded 150 mn (15 crore)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genus Power management, Q4 FY26 earnings call, 19-May-2026: "total consumer base ... 31 to 32 crore, with 15 crore already tendered and 7 crore installed"; tenders for a further 9 crore expected in FY27. Consistent with trajectory: NSGM dashboard showed awarded = 13,80,22,912 (138.02 mn) of 22,23,54,490 sanctioned in early 2025 (the '138 mn / 62%' in the 04-Mar-25 sheet, also cited by Prayas), and CareEdge reported 10.9 crore awarded as of Mar-2024. Note: 15 crore is management commentary, not an official NSGM publication.</t>
   </si>
   <si>
     <t xml:space="preserve">State installed figures</t>
@@ -576,27 +576,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -604,59 +608,55 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -818,22 +818,26 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -882,8 +886,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="66550367"/>
-        <c:axId val="76082649"/>
+        <c:axId val="86120884"/>
+        <c:axId val="84040801"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -918,22 +922,26 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -992,17 +1000,17 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="66550367"/>
-        <c:axId val="76082649"/>
+        <c:axId val="86120884"/>
+        <c:axId val="84040801"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="66550367"/>
+        <c:axId val="86120884"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1028,7 +1036,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76082649"/>
+        <c:crossAx val="84040801"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1036,7 +1044,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76082649"/>
+        <c:axId val="84040801"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1052,7 +1060,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1078,7 +1086,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66550367"/>
+        <c:crossAx val="86120884"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1200,22 +1208,26 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1338,22 +1350,26 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1438,17 +1454,17 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65386420"/>
-        <c:axId val="80838517"/>
+        <c:axId val="34354655"/>
+        <c:axId val="44897"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65386420"/>
+        <c:axId val="34354655"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1474,7 +1490,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80838517"/>
+        <c:crossAx val="44897"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1482,7 +1498,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80838517"/>
+        <c:axId val="44897"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1498,7 +1514,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1524,7 +1540,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65386420"/>
+        <c:crossAx val="34354655"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1679,80 +1695,96 @@
             <c:dLbl>
               <c:idx val="0"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="bestFit"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="bestFit"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
           </c:dLbls>
           <c:cat>
@@ -1852,9 +1884,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>126720</xdr:colOff>
+      <xdr:colOff>126360</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>18360</xdr:rowOff>
+      <xdr:rowOff>18000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1862,8 +1894,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="14538240" y="571680"/>
-        <a:ext cx="4679640" cy="2699640"/>
+        <a:off x="14538240" y="566640"/>
+        <a:ext cx="4679280" cy="2699280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1882,9 +1914,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>48960</xdr:colOff>
+      <xdr:colOff>48600</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>7560</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1892,8 +1924,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="14538240" y="3619440"/>
-        <a:ext cx="6119640" cy="2879640"/>
+        <a:off x="14538240" y="3614040"/>
+        <a:ext cx="6119280" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1912,9 +1944,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>165600</xdr:colOff>
+      <xdr:colOff>165240</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>18360</xdr:rowOff>
+      <xdr:rowOff>18000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1922,8 +1954,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="14538240" y="7429680"/>
-        <a:ext cx="3959640" cy="2699640"/>
+        <a:off x="14538240" y="7424640"/>
+        <a:ext cx="3959280" cy="2699280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2119,150 +2151,150 @@
   <dimension ref="B1:G61"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>27.7</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <f aca="false">C7-C6</f>
         <v>9.7</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="10" t="n">
         <f aca="false">(C7-C6)/C6</f>
         <v>0.538888888888889</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>49.3</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">C8-C7</f>
         <v>21.6</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="10" t="n">
         <f aca="false">(C8-C7)/C7</f>
         <v>0.779783393501805</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>72.4</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">C9-C8</f>
         <v>23.1</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="10" t="n">
         <f aca="false">(C9-C8)/C8</f>
         <v>0.468559837728195</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>222</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="11" t="n">
         <v>72.4</v>
       </c>
       <c r="G14" s="13" t="n">
@@ -2270,11 +2302,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="14" t="n">
@@ -2290,11 +2322,11 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D16" s="16" t="n">
@@ -2314,86 +2346,86 @@
         <v>792000</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <f aca="false">E14/D14</f>
         <v>0.675675675675676</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="5" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="10" t="n">
         <f aca="false">F14/D14</f>
         <v>0.326126126126126</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="5" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="9" t="n">
         <f aca="false">F14</f>
         <v>72.4</v>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="10" t="n">
         <f aca="false">C22/$D$14</f>
         <v>0.326126126126126</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="5" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="9" t="n">
         <f aca="false">E14-F14</f>
         <v>77.6</v>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="10" t="n">
         <f aca="false">C23/$D$14</f>
         <v>0.34954954954955</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="5" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="9" t="n">
         <f aca="false">D14-E14</f>
         <v>72</v>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="10" t="n">
         <f aca="false">C24/$D$14</f>
         <v>0.324324324324324</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
         <v>36</v>
       </c>
@@ -2406,56 +2438,56 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="3" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="4" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="5" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="11" t="n">
         <v>197.9</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="5" t="s">
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>5.253</v>
       </c>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="5" t="s">
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="6" t="s">
         <v>44</v>
       </c>
       <c r="C31" s="20" t="n">
         <v>0.205</v>
       </c>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="15" t="s">
         <v>45</v>
       </c>
@@ -2463,77 +2495,77 @@
         <f aca="false">SUM(C29:C31)</f>
         <v>203.358</v>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="D32" s="11" t="n">
         <v>57.3</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="5" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="8" t="n">
+      <c r="C33" s="6"/>
+      <c r="D33" s="9" t="n">
         <f aca="false">F14-D32</f>
         <v>15.1</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E33" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="5" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6" t="n">
+      <c r="C34" s="6"/>
+      <c r="D34" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="4" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="5" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C38" s="10" t="n">
+      <c r="C38" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="D38" s="10" t="n">
+      <c r="D38" s="11" t="n">
         <v>6.5</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="E38" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F38" s="9" t="n">
+      <c r="F38" s="10" t="n">
         <f aca="false">D38/C38</f>
         <v>0.209677419354839</v>
       </c>
@@ -2541,20 +2573,20 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="5" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="10" t="n">
+      <c r="C39" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="D39" s="10" t="n">
+      <c r="D39" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F39" s="9" t="n">
+      <c r="F39" s="10" t="n">
         <f aca="false">D39/C39</f>
         <v>0.00333333333333333</v>
       </c>
@@ -2562,20 +2594,20 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="5" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="10" t="n">
+      <c r="C40" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="D40" s="10" t="n">
+      <c r="D40" s="11" t="n">
         <v>7.4</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F40" s="9" t="n">
+      <c r="F40" s="10" t="n">
         <f aca="false">D40/C40</f>
         <v>0.308333333333333</v>
       </c>
@@ -2583,38 +2615,38 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="5" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C41" s="10" t="n">
+      <c r="C41" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="7" t="s">
+      <c r="E41" s="6"/>
+      <c r="F41" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G41" s="21" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="5" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="10" t="n">
+      <c r="C42" s="11" t="n">
         <v>17.2</v>
       </c>
-      <c r="D42" s="10" t="n">
+      <c r="D42" s="11" t="n">
         <v>8.2</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F42" s="9" t="n">
+      <c r="F42" s="10" t="n">
         <f aca="false">D42/C42</f>
         <v>0.476744186046512</v>
       </c>
@@ -2622,69 +2654,69 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="5" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C43" s="10" t="n">
+      <c r="C43" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E43" s="5"/>
-      <c r="F43" s="7" t="s">
+      <c r="E43" s="6"/>
+      <c r="F43" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G43" s="21"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C44" s="10" t="n">
+      <c r="C44" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E44" s="5"/>
-      <c r="F44" s="7" t="s">
+      <c r="E44" s="6"/>
+      <c r="F44" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G44" s="21"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="5" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C45" s="10" t="n">
+      <c r="C45" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="D45" s="6" t="n">
+      <c r="D45" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F45" s="9" t="n">
+      <c r="F45" s="10" t="n">
         <f aca="false">D45/C45</f>
         <v>0.0769230769230769</v>
       </c>
       <c r="G45" s="21"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="5" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C46" s="10" t="n">
+      <c r="C46" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="D46" s="10" t="n">
+      <c r="D46" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E46" s="5"/>
-      <c r="F46" s="9" t="n">
+      <c r="E46" s="6"/>
+      <c r="F46" s="10" t="n">
         <f aca="false">D46/C46</f>
         <v>0</v>
       </c>
@@ -2692,36 +2724,36 @@
         <v>73</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="5" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C47" s="10" t="n">
+      <c r="C47" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E47" s="5"/>
-      <c r="F47" s="7" t="s">
+      <c r="E47" s="6"/>
+      <c r="F47" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G47" s="21"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="5" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C48" s="10" t="n">
+      <c r="C48" s="11" t="n">
         <v>3.3</v>
       </c>
-      <c r="D48" s="10" t="n">
+      <c r="D48" s="11" t="n">
         <v>3.3</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="E48" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="F48" s="9" t="n">
+      <c r="F48" s="10" t="n">
         <f aca="false">D48/C48</f>
         <v>1</v>
       </c>
@@ -2729,23 +2761,23 @@
         <v>77</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="5" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="10" t="n">
+      <c r="C49" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="7" t="s">
+      <c r="D49" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="7" t="s">
+      <c r="E49" s="6"/>
+      <c r="F49" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G49" s="21"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="15" t="s">
         <v>79</v>
       </c>
@@ -2758,70 +2790,70 @@
         <v>26.5</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="3" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B52" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="4" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="D53" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E53" s="4" t="s">
+      <c r="E53" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F53" s="4" t="s">
+      <c r="F53" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="5" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C54" s="10" t="n">
+      <c r="C54" s="11" t="n">
         <v>27.5</v>
       </c>
-      <c r="D54" s="10" t="n">
+      <c r="D54" s="11" t="n">
         <v>240.2</v>
       </c>
-      <c r="E54" s="10" t="n">
+      <c r="E54" s="11" t="n">
         <v>10.4</v>
       </c>
       <c r="F54" s="21" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="5" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C55" s="10" t="n">
+      <c r="C55" s="11" t="n">
         <v>24.6</v>
       </c>
-      <c r="D55" s="10" t="n">
+      <c r="D55" s="11" t="n">
         <v>295.2</v>
       </c>
-      <c r="E55" s="10" t="n">
+      <c r="E55" s="11" t="n">
         <v>13.4</v>
       </c>
       <c r="F55" s="21" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="5" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C56" s="10" t="n">
+      <c r="C56" s="11" t="n">
         <v>7.6</v>
       </c>
-      <c r="D56" s="10" t="n">
+      <c r="D56" s="11" t="n">
         <v>76</v>
       </c>
       <c r="E56" s="22" t="s">
@@ -2831,14 +2863,14 @@
         <v>91</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="5" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B57" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C57" s="10" t="n">
+      <c r="C57" s="11" t="n">
         <v>5.2</v>
       </c>
-      <c r="D57" s="10" t="n">
+      <c r="D57" s="11" t="n">
         <v>61.8</v>
       </c>
       <c r="E57" s="22" t="s">
@@ -2848,8 +2880,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="5" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C58" s="22" t="s">
@@ -2865,8 +2897,8 @@
         <v>95</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="5" t="s">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B59" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C59" s="22" t="s">
@@ -2882,8 +2914,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="2" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B61" s="3" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2907,11 +2939,11 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
         <v>99</v>
       </c>
@@ -2919,7 +2951,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
         <v>101</v>
       </c>
@@ -2927,7 +2959,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
         <v>103</v>
       </c>
@@ -2935,7 +2967,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
         <v>105</v>
       </c>
@@ -2943,7 +2975,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
         <v>107</v>
       </c>
@@ -2951,7 +2983,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
         <v>109</v>
       </c>
@@ -2959,7 +2991,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
         <v>111</v>
       </c>
@@ -2967,7 +2999,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
         <v>113</v>
       </c>
@@ -2975,7 +3007,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="24" t="s">
         <v>115</v>
       </c>
@@ -2983,7 +3015,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
         <v>117</v>
       </c>
@@ -2991,7 +3023,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
         <v>119</v>
       </c>
@@ -2999,7 +3031,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
         <v>121</v>
       </c>
@@ -3007,7 +3039,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
         <v>123</v>
       </c>

</xml_diff>

<commit_message>
Update awarded to 156 mn per Genus Q4FY26 call transcript; add call-data sheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Consumer_Metering_Status_Aug2026.xlsx
+++ b/Smart_Consumer_Metering_Status_Aug2026.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Sources &amp; Notes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Genus Q4FY26 Call" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="222">
   <si>
     <t xml:space="preserve">Smart Consumer Metering Status as on 20-Aug-2026</t>
   </si>
@@ -284,7 +285,7 @@
     <t xml:space="preserve">Genus Power (incl. SPVs/GIC JV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Order book Rs.24,020 cr (Jun-26); crossed 1 crore installed Feb-26 across 9 states; targets +1 crore in FY27</t>
+    <t xml:space="preserve">Per Q4FY26 call transcript (19-May-26): order book Rs.25,173 cr incl. SPVs/GIC platform; 24 AMISP projects all OGL, awarded base 3.61 cr meters; crossed 1 cr installed under RDSS (Q&amp;A: 87 lakh own-RDSS, ~30 lakh in Q4); targets &gt;1 cr installs &amp; Rs.6,000-6,500 cr revenue in FY27; capacity 1.8 cr meters/yr</t>
   </si>
   <si>
     <t xml:space="preserve">Adani Energy Solutions (AESL)</t>
@@ -344,10 +345,10 @@
     <t xml:space="preserve">Nov-24: 16.8 mn (NSGM); Mar-25: 24.0 mn (NSGM via tndindia); mid-25: ~27.7 mn (indiasmartgrid.org); 15-Nov-25: 47.6 mn (Mercom India); 11-Dec-25: 49.3 mn, 1.6 cr prepaid (Power Minister, newsonair.gov.in); 15-Feb-26: 58.3 mn @ ~1.35 lakh/day (PFI/pfie.com); 30-Jun-26: 72.4 mn (Parliament)</t>
   </si>
   <si>
-    <t xml:space="preserve">Awarded 150 mn (15 crore)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Genus Power management, Q4 FY26 earnings call, 19-May-2026: "total consumer base ... 31 to 32 crore, with 15 crore already tendered and 7 crore installed"; tenders for a further 9 crore expected in FY27. Consistent with trajectory: NSGM dashboard showed awarded = 13,80,22,912 (138.02 mn) of 22,23,54,490 sanctioned in early 2025 (the '138 mn / 62%' in the 04-Mar-25 sheet, also cited by Prayas), and CareEdge reported 10.9 crore awarded as of Mar-2024. Note: 15 crore is management commentary, not an official NSGM publication.</t>
+    <t xml:space="preserve">Awarded 156 mn (15.6 crore)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIMARY SOURCE: Genus Power Q4FY26 earnings call transcript, 19-May-2026 (BSE/NSE filing, provided by user) — prepared remarks: 'only around 15.6 crore meters have so far been tendered'; Q&amp;A: '15 crores has already been tendered and 7 crores has been installed', with a further ~5 crore of tenders live (Haryana/MP/Punjab/TN) and 9 crore expected in FY27. Trajectory check: NSGM dashboard showed 13,80,22,912 (138.02 mn) awarded of 22,23,54,490 sanctioned in early 2025; CareEdge: 10.9 crore awarded Mar-2024.</t>
   </si>
   <si>
     <t xml:space="preserve">State installed figures</t>
@@ -396,6 +397,297 @@
   </si>
   <si>
     <t xml:space="preserve">nsgm.gov.in / pib.gov.in are geo-blocked from this environment (connection reset) — figures compiled from Parliament replies and industry press instead of the live NSGM dashboard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genus Power Q4 &amp; FY26 Earnings Call — 19-May-2026 (transcript filed 26-May-2026). Source: user-provided PDF (BSE/NSE filing).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry: total consumer base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31-32 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To be replaced with smart meters over next 4-5 years (JMD, Q&amp;A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry: tendered so far</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.6 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepared remarks: 'only around 15.6 crore meters have so far been tendered'; Q&amp;A rounds to 15 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry: installed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches official 7.24 crore as of 30-Jun-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry: remaining to install</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24-25 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry: RDSS sanctioned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Program extended till 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tenders live now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~5 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haryana, MP, Punjab, Tamil Nadu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender pipeline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4+ crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More Haryana, Punjab, Delhi; large quantities from West Bengal, Kerala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tenders expected in FY27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4FY26 revenue (standalone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.1,524 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+63% YoY, +36% QoQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4FY26 EBITDA / PAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.284 cr / Rs.181 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+36% / +41% YoY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.4,738 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+94% YoY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.960 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+104% YoY; margin 20.3% (+102 bps)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 PAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.605 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+106% YoY; margin 12.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order book (31-Mar-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.25,173 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net of taxes, incl. all SPVs &amp; GIC platform; concessions 8-9 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order book split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23,000 + 2,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.23,000 cr platform (Rs.16,000 cr capex + ~Rs.7,000 cr opex/O&amp;M); Rs.2,000 cr exports/gas/water/other AMISPs/utilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMISP projects / awarded base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 / 3.61 crore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 24 projects Operational-Go-Live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meters installed under RDSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 crore+ crossed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q&amp;A: 87 lakh under RDSS program; ~30 lakh installed in Q4FY26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturing capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;1.8 crore/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'exceeding 18 million meters annually'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22-23% / &gt;30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As AMISP / as meter manufacturer + AMISP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 guidance: revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.6,000-6,500 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 guidance: EBITDA margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~18%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.5pp: RM/chips/forex; fixed-price contracts, no pass-through; hardware ~45-50% of platform book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 guidance: installs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;1 crore meters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27 capex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.10-20 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routine only (dies &amp; molds)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O&amp;M revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.150 cr -&gt; Rs.800-900 cr/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 -&gt; within 2-3 yrs, sustained 5-7 yrs, on current order book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.1,573 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs Rs.605 cr Mar-25; peak expected Rs.1,900-2,000 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash &amp; equivalents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.719 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FDs &amp; current investments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIC platform (Gemstar) investment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.487 cr done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genus 26% / GIC 74%; further Rs.600-700 cr over FY27-Q1FY29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working capital days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">343 -&gt; 274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debtors 187-&gt;89, inventory 127-&gt;104; another 50-75 day cut expected FY27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash flow outlook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive from FY28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~Breakeven/slightly negative by end-FY27; positive from Q1-Q2 FY28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gas meters opportunity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 crore / Rs.35,000-36,000 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mandated over 3-4 yrs; Genus to participate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exports target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.500 cr in 2-3 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Australia go-live expected in 3-6 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R&amp;D team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~300 device + ~250 software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HES/MDM/WFM in-house; proprietary interoperable RF mesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IntelliSmart bid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision rests with GIC as platform majority owner</t>
   </si>
 </sst>
 </file>
@@ -571,7 +863,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -673,6 +965,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -886,8 +1198,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86120884"/>
-        <c:axId val="84040801"/>
+        <c:axId val="79530242"/>
+        <c:axId val="43574182"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1000,11 +1312,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="86120884"/>
-        <c:axId val="84040801"/>
+        <c:axId val="79530242"/>
+        <c:axId val="43574182"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="86120884"/>
+        <c:axId val="79530242"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1036,7 +1348,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84040801"/>
+        <c:crossAx val="43574182"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1044,7 +1356,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84040801"/>
+        <c:axId val="43574182"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1086,7 +1398,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86120884"/>
+        <c:crossAx val="79530242"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1454,11 +1766,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="34354655"/>
-        <c:axId val="44897"/>
+        <c:axId val="89317091"/>
+        <c:axId val="22422952"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34354655"/>
+        <c:axId val="89317091"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1490,7 +1802,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44897"/>
+        <c:crossAx val="22422952"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1498,7 +1810,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44897"/>
+        <c:axId val="22422952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1540,7 +1852,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34354655"/>
+        <c:crossAx val="89317091"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1814,10 +2126,10 @@
                   <c:v>72.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77.6</c:v>
+                  <c:v>83.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>72</c:v>
+                  <c:v>66</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1884,9 +2196,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>126360</xdr:colOff>
+      <xdr:colOff>126000</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1895,7 +2207,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="566640"/>
-        <a:ext cx="4679280" cy="2699280"/>
+        <a:ext cx="4678920" cy="2698920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1914,9 +2226,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>48600</xdr:colOff>
+      <xdr:colOff>48240</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>7200</xdr:rowOff>
+      <xdr:rowOff>6840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1925,7 +2237,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="3614040"/>
-        <a:ext cx="6119280" cy="2879640"/>
+        <a:ext cx="6118920" cy="2879280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1944,9 +2256,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>165240</xdr:colOff>
+      <xdr:colOff>164880</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1955,7 +2267,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="7424640"/>
-        <a:ext cx="3959280" cy="2699280"/>
+        <a:ext cx="3958920" cy="2698920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2292,14 +2604,14 @@
         <v>222</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F14" s="11" t="n">
         <v>72.4</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">D14-E14</f>
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2647,7 @@
       </c>
       <c r="E16" s="16" t="n">
         <f aca="false">E14*E15</f>
-        <v>1650000</v>
+        <v>1716000</v>
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">F14*F15</f>
@@ -2343,7 +2655,7 @@
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">G14*G15</f>
-        <v>792000</v>
+        <v>726000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2355,7 +2667,7 @@
       </c>
       <c r="D17" s="10" t="n">
         <f aca="false">E14/D14</f>
-        <v>0.675675675675676</v>
+        <v>0.702702702702703</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2405,11 +2717,11 @@
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">E14-F14</f>
-        <v>77.6</v>
+        <v>83.6</v>
       </c>
       <c r="D23" s="10" t="n">
         <f aca="false">C23/$D$14</f>
-        <v>0.34954954954955</v>
+        <v>0.376576576576577</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2418,11 +2730,11 @@
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">D14-E14</f>
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">C24/$D$14</f>
-        <v>0.324324324324324</v>
+        <v>0.297297297297297</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2817,13 +3129,13 @@
         <v>86</v>
       </c>
       <c r="C54" s="11" t="n">
-        <v>27.5</v>
+        <v>36.1</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>240.2</v>
+        <v>251.7</v>
       </c>
       <c r="E54" s="11" t="n">
-        <v>10.4</v>
+        <v>10</v>
       </c>
       <c r="F54" s="21" t="s">
         <v>87</v>
@@ -3056,4 +3368,399 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="78"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="26" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="30"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" s="30"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>177</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="C23" s="30"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="C25" s="30"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>199</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="B31" s="29" t="s">
+        <v>205</v>
+      </c>
+      <c r="C31" s="30" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="28" t="s">
+        <v>213</v>
+      </c>
+      <c r="B34" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="28" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="C35" s="30" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="B36" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="C36" s="30" t="s">
+        <v>221</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add official state-wise sanctioned/awarded/installed sheet (RS reply 10-Feb-2025 via data.gov.in)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Consumer_Metering_Status_Aug2026.xlsx
+++ b/Smart_Consumer_Metering_Status_Aug2026.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sources &amp; Notes" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Genus Q4FY26 Call" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Statewise S-A-I" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Genus Q4FY26 Call" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="251">
   <si>
     <t xml:space="preserve">Smart Consumer Metering Status as on 20-Aug-2026</t>
   </si>
@@ -319,6 +320,93 @@
   </si>
   <si>
     <t xml:space="preserve">Key meter manufacturers: Genus Power, Secure Meters, HPL Electric, Schneider Electric, Polaris Smart Metering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State/UT-wise Smart Meters under RDSS — Sanctioned / Awarded / Installed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official source: Rajya Sabha Unstarred Question reply, 10-Feb-2025 (Ministry of Power), via data.gov.in API (resource da474c10-b5dc-4e65-b5af-7687ac3079f1). RDSS meters only (consumer + DT + feeder) — Bihar's large pre-RDSS/state-scheme rollout and Haryana/Karnataka/Telangana/Odisha (no RDSS metering sanction) are outside this table. 'Latest installed' column = newer all-scheme press figures where available (dates noted).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State/UT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awarded %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installed %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest installed (mn, all schemes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15-Nov-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02-Dec-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-Mar-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chhattisgarh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andhra Pradesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Himachal Pradesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uttarakhand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jammu and Kashmir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jharkhand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tripura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meghalaya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puducherry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nagaland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arunachal Pradesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mizoram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manipur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sikkim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andaman and Nicobar Islands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delhi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (sum of states)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All India Total (as printed in reply)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Later all-India milestones for context: installed 49.3 mn (11-Dec-25, Minister), 72.4 mn total / 57.3 mn RDSS (30-Jun-26, Parliament); awarded/tendered ~156 mn (Genus Q4FY26 call, 19-May-26).</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -702,7 +790,7 @@
     <numFmt numFmtId="168" formatCode="#,##0"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -780,6 +868,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -863,7 +958,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -956,19 +1051,11 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -980,11 +1067,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1198,8 +1329,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="79530242"/>
-        <c:axId val="43574182"/>
+        <c:axId val="363920"/>
+        <c:axId val="14935987"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1312,11 +1443,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="79530242"/>
-        <c:axId val="43574182"/>
+        <c:axId val="363920"/>
+        <c:axId val="14935987"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79530242"/>
+        <c:axId val="363920"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1348,7 +1479,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43574182"/>
+        <c:crossAx val="14935987"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1356,7 +1487,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43574182"/>
+        <c:axId val="14935987"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1398,7 +1529,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79530242"/>
+        <c:crossAx val="363920"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1766,11 +1897,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="89317091"/>
-        <c:axId val="22422952"/>
+        <c:axId val="711310"/>
+        <c:axId val="33240847"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="89317091"/>
+        <c:axId val="711310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1802,7 +1933,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22422952"/>
+        <c:crossAx val="33240847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1810,7 +1941,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22422952"/>
+        <c:axId val="33240847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1852,7 +1983,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89317091"/>
+        <c:crossAx val="711310"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2196,9 +2327,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>126000</xdr:colOff>
+      <xdr:colOff>125640</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>17640</xdr:rowOff>
+      <xdr:rowOff>17280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2207,7 +2338,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="566640"/>
-        <a:ext cx="4678920" cy="2698920"/>
+        <a:ext cx="4678560" cy="2698560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2226,9 +2357,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>48240</xdr:colOff>
+      <xdr:colOff>47880</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2237,7 +2368,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="3614040"/>
-        <a:ext cx="6118920" cy="2879280"/>
+        <a:ext cx="6118560" cy="2878920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2256,9 +2387,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>164880</xdr:colOff>
+      <xdr:colOff>164520</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>17640</xdr:rowOff>
+      <xdr:rowOff>17280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2267,7 +2398,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="7424640"/>
-        <a:ext cx="3958920" cy="2698920"/>
+        <a:ext cx="3958560" cy="2698560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3248,118 +3379,810 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="B1:I37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="23" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="24" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="C5" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="25" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
+      <c r="G5" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="H5" s="25" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
+      <c r="I5" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>30490774</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <f aca="false">IF(C6=0,"",D6/C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="28" t="n">
+        <f aca="false">IF(C6=0,"",E6/C6)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="29"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>28526731</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>28526730</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>858147</v>
+      </c>
+      <c r="F7" s="28" t="n">
+        <f aca="false">IF(C7=0,"",D7/C7)</f>
+        <v>0.99999996494516</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <f aca="false">IF(C7=0,"",E7/C7)</f>
+        <v>0.0300822060543846</v>
+      </c>
+      <c r="H7" s="31" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="I7" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="25" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>24004866</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>25273775</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>696405</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <f aca="false">IF(C8=0,"",D8/C8)</f>
+        <v>1.05286049086881</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <f aca="false">IF(C8=0,"",E8/C8)</f>
+        <v>0.029010993021165</v>
+      </c>
+      <c r="H8" s="31" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="I8" s="26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>21035262</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>4031566</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>178681</v>
+      </c>
+      <c r="F9" s="28" t="n">
+        <f aca="false">IF(C9=0,"",D9/C9)</f>
+        <v>0.191657512989379</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <f aca="false">IF(C9=0,"",E9/C9)</f>
+        <v>0.00849435581073343</v>
+      </c>
+      <c r="H9" s="29"/>
+      <c r="I9" s="30"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <v>16787587</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>11071687</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>425818</v>
+      </c>
+      <c r="F10" s="28" t="n">
+        <f aca="false">IF(C10=0,"",D10/C10)</f>
+        <v>0.659516284264082</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <f aca="false">IF(C10=0,"",E10/C10)</f>
+        <v>0.0253650509748661</v>
+      </c>
+      <c r="H10" s="29"/>
+      <c r="I10" s="30"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>14736692</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>14754023</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>11416</v>
+      </c>
+      <c r="F11" s="28" t="n">
+        <f aca="false">IF(C11=0,"",D11/C11)</f>
+        <v>1.00117604412171</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <f aca="false">IF(C11=0,"",E11/C11)</f>
+        <v>0.00077466503337384</v>
+      </c>
+      <c r="H11" s="29"/>
+      <c r="I11" s="30"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="27" t="n">
+        <v>13429206</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>5490509</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>1366302</v>
+      </c>
+      <c r="F12" s="28" t="n">
+        <f aca="false">IF(C12=0,"",D12/C12)</f>
+        <v>0.408848371229096</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <f aca="false">IF(C12=0,"",E12/C12)</f>
+        <v>0.101741085809541</v>
+      </c>
+      <c r="H12" s="31" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="I12" s="26" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="27" t="n">
+        <v>13383001</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>291690</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="28" t="n">
+        <f aca="false">IF(C13=0,"",D13/C13)</f>
+        <v>0.021795559904688</v>
+      </c>
+      <c r="G13" s="28" t="n">
+        <f aca="false">IF(C13=0,"",E13/C13)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="29"/>
+      <c r="I13" s="30"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="27" t="n">
+        <v>8981414</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="28" t="n">
+        <f aca="false">IF(C14=0,"",D14/C14)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="28" t="n">
+        <f aca="false">IF(C14=0,"",E14/C14)</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="29"/>
+      <c r="I14" s="30"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="27" t="n">
+        <v>6445127</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>6558446</v>
+      </c>
+      <c r="E15" s="27" t="n">
+        <v>2520475</v>
+      </c>
+      <c r="F15" s="28" t="n">
+        <f aca="false">IF(C15=0,"",D15/C15)</f>
+        <v>1.01758212056954</v>
+      </c>
+      <c r="G15" s="28" t="n">
+        <f aca="false">IF(C15=0,"",E15/C15)</f>
+        <v>0.391066770290174</v>
+      </c>
+      <c r="H15" s="31" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="I15" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="25" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="26" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="C16" s="27" t="n">
+        <v>6179479</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>7345604</v>
+      </c>
+      <c r="E16" s="27" t="n">
+        <v>1046898</v>
+      </c>
+      <c r="F16" s="28" t="n">
+        <f aca="false">IF(C16=0,"",D16/C16)</f>
+        <v>1.18870927468157</v>
+      </c>
+      <c r="G16" s="28" t="n">
+        <f aca="false">IF(C16=0,"",E16/C16)</f>
+        <v>0.169415253292389</v>
+      </c>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="C17" s="27" t="n">
+        <v>5919344</v>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>5981561</v>
+      </c>
+      <c r="E17" s="27" t="n">
+        <v>823382</v>
+      </c>
+      <c r="F17" s="28" t="n">
+        <f aca="false">IF(C17=0,"",D17/C17)</f>
+        <v>1.01051079308788</v>
+      </c>
+      <c r="G17" s="28" t="n">
+        <f aca="false">IF(C17=0,"",E17/C17)</f>
+        <v>0.139100211104474</v>
+      </c>
+      <c r="H17" s="29"/>
+      <c r="I17" s="30"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="26" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="C18" s="27" t="n">
+        <v>2841908</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>934409</v>
+      </c>
+      <c r="E18" s="27" t="n">
+        <v>103524</v>
+      </c>
+      <c r="F18" s="28" t="n">
+        <f aca="false">IF(C18=0,"",D18/C18)</f>
+        <v>0.328796357939807</v>
+      </c>
+      <c r="G18" s="28" t="n">
+        <f aca="false">IF(C18=0,"",E18/C18)</f>
+        <v>0.0364276394591239</v>
+      </c>
+      <c r="H18" s="29"/>
+      <c r="I18" s="30"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="27" t="n">
+        <v>2607153</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>2598542</v>
+      </c>
+      <c r="E19" s="27" t="n">
+        <v>1861464</v>
+      </c>
+      <c r="F19" s="28" t="n">
+        <f aca="false">IF(C19=0,"",D19/C19)</f>
+        <v>0.996697163534323</v>
+      </c>
+      <c r="G19" s="28" t="n">
+        <f aca="false">IF(C19=0,"",E19/C19)</f>
+        <v>0.713983414091923</v>
+      </c>
+      <c r="H19" s="31" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="C20" s="27" t="n">
+        <v>1649684</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <v>1649684</v>
+      </c>
+      <c r="E20" s="27" t="n">
+        <v>12720</v>
+      </c>
+      <c r="F20" s="28" t="n">
+        <f aca="false">IF(C20=0,"",D20/C20)</f>
+        <v>1</v>
+      </c>
+      <c r="G20" s="28" t="n">
+        <f aca="false">IF(C20=0,"",E20/C20)</f>
+        <v>0.00771056759961302</v>
+      </c>
+      <c r="H20" s="29"/>
+      <c r="I20" s="30"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="26" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
+      <c r="C21" s="27" t="n">
+        <v>1497690</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>1490727</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>14707</v>
+      </c>
+      <c r="F21" s="28" t="n">
+        <f aca="false">IF(C21=0,"",D21/C21)</f>
+        <v>0.995350840294053</v>
+      </c>
+      <c r="G21" s="28" t="n">
+        <f aca="false">IF(C21=0,"",E21/C21)</f>
+        <v>0.00981978914194526</v>
+      </c>
+      <c r="H21" s="29"/>
+      <c r="I21" s="30"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="C22" s="27" t="n">
+        <v>1362044</v>
+      </c>
+      <c r="D22" s="27" t="n">
+        <v>1362044</v>
+      </c>
+      <c r="E22" s="27" t="n">
+        <v>15680</v>
+      </c>
+      <c r="F22" s="28" t="n">
+        <f aca="false">IF(C22=0,"",D22/C22)</f>
+        <v>1</v>
+      </c>
+      <c r="G22" s="28" t="n">
+        <f aca="false">IF(C22=0,"",E22/C22)</f>
+        <v>0.0115121097409482</v>
+      </c>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="26" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+      <c r="C23" s="27" t="n">
+        <v>750356</v>
+      </c>
+      <c r="D23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="28" t="n">
+        <f aca="false">IF(C23=0,"",D23/C23)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="28" t="n">
+        <f aca="false">IF(C23=0,"",E23/C23)</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="29"/>
+      <c r="I23" s="30"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="C24" s="27" t="n">
+        <v>562870</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <v>427013</v>
+      </c>
+      <c r="E24" s="27" t="n">
+        <v>3694</v>
+      </c>
+      <c r="F24" s="28" t="n">
+        <f aca="false">IF(C24=0,"",D24/C24)</f>
+        <v>0.758635208840407</v>
+      </c>
+      <c r="G24" s="28" t="n">
+        <f aca="false">IF(C24=0,"",E24/C24)</f>
+        <v>0.00656279425089275</v>
+      </c>
+      <c r="H24" s="29"/>
+      <c r="I24" s="30"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="26" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+      <c r="C25" s="27" t="n">
+        <v>472743</v>
+      </c>
+      <c r="D25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="28" t="n">
+        <f aca="false">IF(C25=0,"",D25/C25)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="28" t="n">
+        <f aca="false">IF(C25=0,"",E25/C25)</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="29"/>
+      <c r="I25" s="30"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="C26" s="27" t="n">
+        <v>407052</v>
+      </c>
+      <c r="D26" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="28" t="n">
+        <f aca="false">IF(C26=0,"",D26/C26)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="28" t="n">
+        <f aca="false">IF(C26=0,"",E26/C26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="29"/>
+      <c r="I26" s="30"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="26" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="C27" s="27" t="n">
+        <v>323878</v>
+      </c>
+      <c r="D27" s="27" t="n">
+        <v>323878</v>
+      </c>
+      <c r="E27" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="28" t="n">
+        <f aca="false">IF(C27=0,"",D27/C27)</f>
+        <v>1</v>
+      </c>
+      <c r="G27" s="28" t="n">
+        <f aca="false">IF(C27=0,"",E27/C27)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="29"/>
+      <c r="I27" s="30"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="C28" s="27" t="n">
+        <v>298250</v>
+      </c>
+      <c r="D28" s="27" t="n">
+        <v>298250</v>
+      </c>
+      <c r="E28" s="27" t="n">
+        <v>276</v>
+      </c>
+      <c r="F28" s="28" t="n">
+        <f aca="false">IF(C28=0,"",D28/C28)</f>
+        <v>1</v>
+      </c>
+      <c r="G28" s="28" t="n">
+        <f aca="false">IF(C28=0,"",E28/C28)</f>
+        <v>0.000925398155909472</v>
+      </c>
+      <c r="H28" s="29"/>
+      <c r="I28" s="30"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="26" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+      <c r="C29" s="27" t="n">
+        <v>292081</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <v>292081</v>
+      </c>
+      <c r="E29" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="28" t="n">
+        <f aca="false">IF(C29=0,"",D29/C29)</f>
+        <v>1</v>
+      </c>
+      <c r="G29" s="28" t="n">
+        <f aca="false">IF(C29=0,"",E29/C29)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="29"/>
+      <c r="I29" s="30"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="C30" s="27" t="n">
+        <v>166208</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>166208</v>
+      </c>
+      <c r="E30" s="27" t="n">
+        <v>628</v>
+      </c>
+      <c r="F30" s="28" t="n">
+        <f aca="false">IF(C30=0,"",D30/C30)</f>
+        <v>1</v>
+      </c>
+      <c r="G30" s="28" t="n">
+        <f aca="false">IF(C30=0,"",E30/C30)</f>
+        <v>0.00377839815171352</v>
+      </c>
+      <c r="H30" s="29"/>
+      <c r="I30" s="30"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="26" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+      <c r="C31" s="27" t="n">
+        <v>148542</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <v>148542</v>
+      </c>
+      <c r="E31" s="27" t="n">
+        <v>11170</v>
+      </c>
+      <c r="F31" s="28" t="n">
+        <f aca="false">IF(C31=0,"",D31/C31)</f>
+        <v>1</v>
+      </c>
+      <c r="G31" s="28" t="n">
+        <f aca="false">IF(C31=0,"",E31/C31)</f>
+        <v>0.0751975872143905</v>
+      </c>
+      <c r="H31" s="29"/>
+      <c r="I31" s="30"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="C32" s="27" t="n">
+        <v>84835</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="28" t="n">
+        <f aca="false">IF(C32=0,"",D32/C32)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="28" t="n">
+        <f aca="false">IF(C32=0,"",E32/C32)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="29"/>
+      <c r="I32" s="30"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="26" t="s">
         <v>124</v>
       </c>
+      <c r="C33" s="27" t="n">
+        <v>3521</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <f aca="false">IF(C33=0,"",D33/C33)</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="28" t="n">
+        <f aca="false">IF(C33=0,"",E33/C33)</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="29"/>
+      <c r="I33" s="30"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" s="33" t="n">
+        <f aca="false">SUM(C6:C33)</f>
+        <v>203388298</v>
+      </c>
+      <c r="D34" s="33" t="n">
+        <f aca="false">SUM(D6:D33)</f>
+        <v>119016969</v>
+      </c>
+      <c r="E34" s="33" t="n">
+        <f aca="false">SUM(E6:E33)</f>
+        <v>9951387</v>
+      </c>
+      <c r="F34" s="28" t="n">
+        <f aca="false">D34/C34</f>
+        <v>0.585171173417263</v>
+      </c>
+      <c r="G34" s="28" t="n">
+        <f aca="false">E34/C34</f>
+        <v>0.0489280214144867</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="27" t="n">
+        <v>203388298</v>
+      </c>
+      <c r="D35" s="27" t="n">
+        <v>119016969</v>
+      </c>
+      <c r="E35" s="27" t="n">
+        <v>9951387</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="34" t="s">
+        <v>127</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:I3"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3375,383 +4198,510 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:C36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="78"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="26" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="B4" s="29" t="s">
+    <row r="1" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="38" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="B3" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
-        <v>130</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
-        <v>136</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="C7" s="30"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
-        <v>138</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
-        <v>147</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" s="30"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>153</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
-        <v>155</v>
-      </c>
-      <c r="B14" s="29" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="B4" s="15" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
+      <c r="C4" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="B15" s="29" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="B5" s="15" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="C5" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="B16" s="29" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="B6" s="15" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
+      <c r="C6" s="39" t="s">
         <v>164</v>
       </c>
-      <c r="B17" s="29" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="B7" s="15" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="C7" s="39"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B8" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="C8" s="39" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B9" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C9" s="39" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B10" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C10" s="39" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B11" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C11" s="39"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
+      <c r="B12" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="C12" s="39" t="s">
         <v>180</v>
       </c>
-      <c r="C22" s="30" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="B13" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="C13" s="39" t="s">
         <v>183</v>
       </c>
-      <c r="C23" s="30"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B14" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C14" s="39" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B15" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="C25" s="30"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
+      <c r="C15" s="39" t="s">
         <v>189</v>
       </c>
-      <c r="B26" s="29" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="B16" s="15" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
+      <c r="C16" s="39" t="s">
         <v>192</v>
       </c>
-      <c r="B27" s="29" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="B17" s="15" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
+      <c r="C17" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="B28" s="29" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="B18" s="15" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
+      <c r="C18" s="39" t="s">
         <v>198</v>
       </c>
-      <c r="B29" s="29" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="C29" s="30" t="s">
+      <c r="B19" s="15" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+      <c r="C19" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="B30" s="29" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="B20" s="15" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="C20" s="39" t="s">
         <v>204</v>
       </c>
-      <c r="B31" s="29" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="B21" s="15" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="C21" s="39" t="s">
         <v>207</v>
       </c>
-      <c r="B32" s="29" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="B22" s="15" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28" t="s">
+      <c r="C22" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="B33" s="29" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="B23" s="15" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
+      <c r="C23" s="39"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B24" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C24" s="39" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="28" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B25" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C25" s="39"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="28" t="s">
+      <c r="B26" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="C26" s="39" t="s">
         <v>220</v>
       </c>
-      <c r="C36" s="30" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>221</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="C27" s="39" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C28" s="39" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="C29" s="39" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="C30" s="39" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="C31" s="39" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="C32" s="39" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="C33" s="39" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="C34" s="39" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="C35" s="39" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="C36" s="39" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add AMISP bidding competitive-intensity data sheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Consumer_Metering_Status_Aug2026.xlsx
+++ b/Smart_Consumer_Metering_Status_Aug2026.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Statewise S-A-I" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Sources &amp; Notes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Genus Q4FY26 Call" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Bidding Intensity" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="309">
   <si>
     <t xml:space="preserve">Smart Consumer Metering Status as on 20-Aug-2026</t>
   </si>
@@ -776,6 +777,180 @@
   </si>
   <si>
     <t xml:space="preserve">Decision rests with GIC as platform majority owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMISP Bidding — Competitive Intensity Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: L1 vs L2 financial bid spreads are NOT public — RFP &amp; AMISP contracts carry confidentiality clauses (Prayas, Apr-2025). Competitive intensity must be read from: (1) award-rate dispersion, (2) PMPM service-charge spread, (3) bidder pools per tender, (4) benchmark-vs-L1 gaps, (5) consolidation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) Award-rate dispersion — single-phase consumer meters, 33 discoms (RDSS dashboard via Prayas, Apr-2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs./meter (10-yr TOTEX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lowest award rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean (right-skewed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Highest (large discoms)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outlier: Sikkim (smallest volume)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max/Min spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.67x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DT meters: Rs.15,962 - 51,660 (median 28,954). Feeder: Rs.14,755 - 1,33,765 (median 48,529; Tripura/Mizoram/HP highest). Select-state single-phase: highest exceeds lowest by 45%, no correlation with volume.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2) PMPM service charge won (= (award rate - subsidy)/93 months) — proxy for how aggressively each state's tender was bid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMPM Rs./meter/month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">West Bengal (lowest = most aggressive)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madhya Pradesh (avg, highest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MP Paschim discom (max)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.8x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3) Tender case studies — bidder pools &amp; outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidders / competition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UP 4 discoms, Round 1 (2022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.85 cr meters, ~Rs.23,000 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adani, GMR, L&amp;T bid all 4; IntelliSmart 2 (3-4 bidders/tender)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrapped: L1 (Adani) quoted ~Rs.10,000/meter vs REC benchmark ~Rs.6,000 — 67% above benchmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UP re-bid (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same pool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PVVNL: IntelliSmart L1 (67 lakh, Apr-23); awards near Rs.9,000/meter level (national median 8,839)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSEDCL Maharashtra (Sep-23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 packages, 1.72+ cr meters, Rs.20,000+ cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple packages split competition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winners: Adani (largest share), NCC, Genus, Montecarlo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chhattisgarh Pkg-2 (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~Rs.1,744 cr / 10 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tata Power L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamil Nadu R1 (2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82 lakh meters, ~Rs.19,000 cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancelled (Adani-linked controversy); re-tendered via PFC Consulting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamil Nadu Phase-2 (Jun-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.45 lakh meters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restricted to 8 empanelled Group-2 entities: Apraava, Adani, Genus, IntelliSmart, GMR, Iskraemeco, Polaris, Montecarlo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidding ongoing; R1 closed 16-Mar-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punjab PSPCL (Jan-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~1 cr meters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSU route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCIL L1 (LoA 30-Jan-26); agreement unsigned as of Jul-26 amid CAPEX-vs-RDSS dispute (~Rs.350 cr implication alleged)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4) Market structure &amp; consolidation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- AMISP market shares (Genus mgmt, Q4FY26 call): Genus ~22-23% as AMISP, &gt;30% as manufacturer+AMISP; AESL order book 24.6 mn meters; IntelliSmart ~Rs.20,000 cr orders (UP/Gujarat/Bihar/Assam); AESL ~Rs.25,000 cr (Maharashtra/Bihar/Assam/AP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Manufacturing: ~10 crore meters/yr capacity; top 8-9 manufacturers hold 70-80% (CareEdge, Mar-25). Genus alone 1.8 crore/yr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Consolidation shrinking the bidder pool: IntelliSmart stake sale (~$400 mn; Adani &amp; GMR in final round); Polaris Smart Metering sale (Adani, Actis, Apraava in round 2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Barriers to entry keep intensity moderate: TOTEX annuity over 93-month O&amp;M, DDF payment security, working-capital drag (Genus WC 274 days FY26), empanelment requirements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Trend: FY27 pipeline of ~9 crore meters of tenders (Genus call) vs 8-10 active AMISPs -&gt; intensity rising in large states, single-bidder risk persists in small/NE states.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sources: Prayas (Energy Group) Apr-2025 (RDSS dashboard compilation); ThePrint 24-Oct-22; T&amp;D India 22-Sep-23 &amp; 15-Jun-26; Tehelka Jul-26; CareEdge Mar-2025; Genus Q4FY26 call transcript; Tata Power release.</t>
   </si>
 </sst>
 </file>
@@ -790,7 +965,7 @@
     <numFmt numFmtId="168" formatCode="#,##0"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -882,6 +1057,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="8.5"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -958,7 +1141,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1051,7 +1234,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1059,43 +1242,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1117,6 +1280,42 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1329,8 +1528,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="363920"/>
-        <c:axId val="14935987"/>
+        <c:axId val="88362268"/>
+        <c:axId val="51747353"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1443,11 +1642,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="363920"/>
-        <c:axId val="14935987"/>
+        <c:axId val="88362268"/>
+        <c:axId val="51747353"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="363920"/>
+        <c:axId val="88362268"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1479,7 +1678,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14935987"/>
+        <c:crossAx val="51747353"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1487,7 +1686,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14935987"/>
+        <c:axId val="51747353"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1529,7 +1728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="363920"/>
+        <c:crossAx val="88362268"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1897,11 +2096,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="711310"/>
-        <c:axId val="33240847"/>
+        <c:axId val="6985815"/>
+        <c:axId val="79293854"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="711310"/>
+        <c:axId val="6985815"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1933,7 +2132,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33240847"/>
+        <c:crossAx val="79293854"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1941,7 +2140,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33240847"/>
+        <c:axId val="79293854"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1983,7 +2182,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="711310"/>
+        <c:crossAx val="6985815"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2327,9 +2526,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>125640</xdr:colOff>
+      <xdr:colOff>125280</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>17280</xdr:rowOff>
+      <xdr:rowOff>16920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2338,7 +2537,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="566640"/>
-        <a:ext cx="4678560" cy="2698560"/>
+        <a:ext cx="4678200" cy="2698200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2357,9 +2556,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>47880</xdr:colOff>
+      <xdr:colOff>47520</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>6480</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2368,7 +2567,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="3614040"/>
-        <a:ext cx="6118560" cy="2878920"/>
+        <a:ext cx="6118200" cy="2878560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2387,9 +2586,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>164520</xdr:colOff>
+      <xdr:colOff>164160</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>17280</xdr:rowOff>
+      <xdr:rowOff>16920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2398,7 +2597,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="7424640"/>
-        <a:ext cx="3958560" cy="2698560"/>
+        <a:ext cx="3958200" cy="2698200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3382,15 +3581,15 @@
   <dimension ref="B1:I37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="23" t="s">
         <v>99</v>
       </c>
@@ -3407,7 +3606,7 @@
       <c r="H2" s="24"/>
       <c r="I2" s="24"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
       <c r="D3" s="24"/>
@@ -3417,765 +3616,765 @@
       <c r="H3" s="24"/>
       <c r="I3" s="24"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="25" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="26" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="14" t="n">
         <v>30490774</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="25" t="n">
         <f aca="false">IF(C6=0,"",D6/C6)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="25" t="n">
         <f aca="false">IF(C6=0,"",E6/C6)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="30"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="26" t="s">
+      <c r="H6" s="26"/>
+      <c r="I6" s="27"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="14" t="n">
         <v>28526731</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="14" t="n">
         <v>28526730</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="14" t="n">
         <v>858147</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="25" t="n">
         <f aca="false">IF(C7=0,"",D7/C7)</f>
         <v>0.99999996494516</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="25" t="n">
         <f aca="false">IF(C7=0,"",E7/C7)</f>
         <v>0.0300822060543846</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="28" t="n">
         <v>6.51</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="26" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="14" t="n">
         <v>24004866</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="14" t="n">
         <v>25273775</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="14" t="n">
         <v>696405</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="25" t="n">
         <f aca="false">IF(C8=0,"",D8/C8)</f>
         <v>1.05286049086881</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="25" t="n">
         <f aca="false">IF(C8=0,"",E8/C8)</f>
         <v>0.029010993021165</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H8" s="28" t="n">
         <v>7.4</v>
       </c>
-      <c r="I8" s="26" t="s">
+      <c r="I8" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="26" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="14" t="n">
         <v>21035262</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="14" t="n">
         <v>4031566</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="14" t="n">
         <v>178681</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="25" t="n">
         <f aca="false">IF(C9=0,"",D9/C9)</f>
         <v>0.191657512989379</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="25" t="n">
         <f aca="false">IF(C9=0,"",E9/C9)</f>
         <v>0.00849435581073343</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="30"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="26" t="s">
+      <c r="H9" s="26"/>
+      <c r="I9" s="27"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="14" t="n">
         <v>16787587</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="14" t="n">
         <v>11071687</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="14" t="n">
         <v>425818</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="25" t="n">
         <f aca="false">IF(C10=0,"",D10/C10)</f>
         <v>0.659516284264082</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="25" t="n">
         <f aca="false">IF(C10=0,"",E10/C10)</f>
         <v>0.0253650509748661</v>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="30"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="26" t="s">
+      <c r="H10" s="26"/>
+      <c r="I10" s="27"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="14" t="n">
         <v>14736692</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="14" t="n">
         <v>14754023</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="14" t="n">
         <v>11416</v>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="25" t="n">
         <f aca="false">IF(C11=0,"",D11/C11)</f>
         <v>1.00117604412171</v>
       </c>
-      <c r="G11" s="28" t="n">
+      <c r="G11" s="25" t="n">
         <f aca="false">IF(C11=0,"",E11/C11)</f>
         <v>0.00077466503337384</v>
       </c>
-      <c r="H11" s="29"/>
-      <c r="I11" s="30"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="26" t="s">
+      <c r="H11" s="26"/>
+      <c r="I11" s="27"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="14" t="n">
         <v>13429206</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="14" t="n">
         <v>5490509</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="14" t="n">
         <v>1366302</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="25" t="n">
         <f aca="false">IF(C12=0,"",D12/C12)</f>
         <v>0.408848371229096</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="25" t="n">
         <f aca="false">IF(C12=0,"",E12/C12)</f>
         <v>0.101741085809541</v>
       </c>
-      <c r="H12" s="31" t="n">
+      <c r="H12" s="28" t="n">
         <v>1.01</v>
       </c>
-      <c r="I12" s="26" t="s">
+      <c r="I12" s="6" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="26" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="14" t="n">
         <v>13383001</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="14" t="n">
         <v>291690</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="25" t="n">
         <f aca="false">IF(C13=0,"",D13/C13)</f>
         <v>0.021795559904688</v>
       </c>
-      <c r="G13" s="28" t="n">
+      <c r="G13" s="25" t="n">
         <f aca="false">IF(C13=0,"",E13/C13)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="29"/>
-      <c r="I13" s="30"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="26" t="s">
+      <c r="H13" s="26"/>
+      <c r="I13" s="27"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="14" t="n">
         <v>8981414</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="25" t="n">
         <f aca="false">IF(C14=0,"",D14/C14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="28" t="n">
+      <c r="G14" s="25" t="n">
         <f aca="false">IF(C14=0,"",E14/C14)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="29"/>
-      <c r="I14" s="30"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="26" t="s">
+      <c r="H14" s="26"/>
+      <c r="I14" s="27"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="14" t="n">
         <v>6445127</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="14" t="n">
         <v>6558446</v>
       </c>
-      <c r="E15" s="27" t="n">
+      <c r="E15" s="14" t="n">
         <v>2520475</v>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="25" t="n">
         <f aca="false">IF(C15=0,"",D15/C15)</f>
         <v>1.01758212056954</v>
       </c>
-      <c r="G15" s="28" t="n">
+      <c r="G15" s="25" t="n">
         <f aca="false">IF(C15=0,"",E15/C15)</f>
         <v>0.391066770290174</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H15" s="28" t="n">
         <v>3.28</v>
       </c>
-      <c r="I15" s="26" t="s">
+      <c r="I15" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="26" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="14" t="n">
         <v>6179479</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="14" t="n">
         <v>7345604</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="14" t="n">
         <v>1046898</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="25" t="n">
         <f aca="false">IF(C16=0,"",D16/C16)</f>
         <v>1.18870927468157</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="25" t="n">
         <f aca="false">IF(C16=0,"",E16/C16)</f>
         <v>0.169415253292389</v>
       </c>
-      <c r="H16" s="29"/>
-      <c r="I16" s="30"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="26" t="s">
+      <c r="H16" s="26"/>
+      <c r="I16" s="27"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="27" t="n">
+      <c r="C17" s="14" t="n">
         <v>5919344</v>
       </c>
-      <c r="D17" s="27" t="n">
+      <c r="D17" s="14" t="n">
         <v>5981561</v>
       </c>
-      <c r="E17" s="27" t="n">
+      <c r="E17" s="14" t="n">
         <v>823382</v>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="25" t="n">
         <f aca="false">IF(C17=0,"",D17/C17)</f>
         <v>1.01051079308788</v>
       </c>
-      <c r="G17" s="28" t="n">
+      <c r="G17" s="25" t="n">
         <f aca="false">IF(C17=0,"",E17/C17)</f>
         <v>0.139100211104474</v>
       </c>
-      <c r="H17" s="29"/>
-      <c r="I17" s="30"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="26" t="s">
+      <c r="H17" s="26"/>
+      <c r="I17" s="27"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="27" t="n">
+      <c r="C18" s="14" t="n">
         <v>2841908</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D18" s="14" t="n">
         <v>934409</v>
       </c>
-      <c r="E18" s="27" t="n">
+      <c r="E18" s="14" t="n">
         <v>103524</v>
       </c>
-      <c r="F18" s="28" t="n">
+      <c r="F18" s="25" t="n">
         <f aca="false">IF(C18=0,"",D18/C18)</f>
         <v>0.328796357939807</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="25" t="n">
         <f aca="false">IF(C18=0,"",E18/C18)</f>
         <v>0.0364276394591239</v>
       </c>
-      <c r="H18" s="29"/>
-      <c r="I18" s="30"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="26" t="s">
+      <c r="H18" s="26"/>
+      <c r="I18" s="27"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="27" t="n">
+      <c r="C19" s="14" t="n">
         <v>2607153</v>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D19" s="14" t="n">
         <v>2598542</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="14" t="n">
         <v>1861464</v>
       </c>
-      <c r="F19" s="28" t="n">
+      <c r="F19" s="25" t="n">
         <f aca="false">IF(C19=0,"",D19/C19)</f>
         <v>0.996697163534323</v>
       </c>
-      <c r="G19" s="28" t="n">
+      <c r="G19" s="25" t="n">
         <f aca="false">IF(C19=0,"",E19/C19)</f>
         <v>0.713983414091923</v>
       </c>
-      <c r="H19" s="31" t="n">
+      <c r="H19" s="28" t="n">
         <v>8.24</v>
       </c>
-      <c r="I19" s="26" t="s">
+      <c r="I19" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="26" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="14" t="n">
         <v>1649684</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="14" t="n">
         <v>1649684</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="14" t="n">
         <v>12720</v>
       </c>
-      <c r="F20" s="28" t="n">
+      <c r="F20" s="25" t="n">
         <f aca="false">IF(C20=0,"",D20/C20)</f>
         <v>1</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="25" t="n">
         <f aca="false">IF(C20=0,"",E20/C20)</f>
         <v>0.00771056759961302</v>
       </c>
-      <c r="H20" s="29"/>
-      <c r="I20" s="30"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="26" t="s">
+      <c r="H20" s="26"/>
+      <c r="I20" s="27"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C21" s="14" t="n">
         <v>1497690</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D21" s="14" t="n">
         <v>1490727</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="14" t="n">
         <v>14707</v>
       </c>
-      <c r="F21" s="28" t="n">
+      <c r="F21" s="25" t="n">
         <f aca="false">IF(C21=0,"",D21/C21)</f>
         <v>0.995350840294053</v>
       </c>
-      <c r="G21" s="28" t="n">
+      <c r="G21" s="25" t="n">
         <f aca="false">IF(C21=0,"",E21/C21)</f>
         <v>0.00981978914194526</v>
       </c>
-      <c r="H21" s="29"/>
-      <c r="I21" s="30"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="26" t="s">
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C22" s="27" t="n">
+      <c r="C22" s="14" t="n">
         <v>1362044</v>
       </c>
-      <c r="D22" s="27" t="n">
+      <c r="D22" s="14" t="n">
         <v>1362044</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="14" t="n">
         <v>15680</v>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="25" t="n">
         <f aca="false">IF(C22=0,"",D22/C22)</f>
         <v>1</v>
       </c>
-      <c r="G22" s="28" t="n">
+      <c r="G22" s="25" t="n">
         <f aca="false">IF(C22=0,"",E22/C22)</f>
         <v>0.0115121097409482</v>
       </c>
-      <c r="H22" s="29"/>
-      <c r="I22" s="30"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="26" t="s">
+      <c r="H22" s="26"/>
+      <c r="I22" s="27"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C23" s="27" t="n">
+      <c r="C23" s="14" t="n">
         <v>750356</v>
       </c>
-      <c r="D23" s="27" t="n">
+      <c r="D23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="27" t="n">
+      <c r="E23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="28" t="n">
+      <c r="F23" s="25" t="n">
         <f aca="false">IF(C23=0,"",D23/C23)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="28" t="n">
+      <c r="G23" s="25" t="n">
         <f aca="false">IF(C23=0,"",E23/C23)</f>
         <v>0</v>
       </c>
-      <c r="H23" s="29"/>
-      <c r="I23" s="30"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="26" t="s">
+      <c r="H23" s="26"/>
+      <c r="I23" s="27"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C24" s="27" t="n">
+      <c r="C24" s="14" t="n">
         <v>562870</v>
       </c>
-      <c r="D24" s="27" t="n">
+      <c r="D24" s="14" t="n">
         <v>427013</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E24" s="14" t="n">
         <v>3694</v>
       </c>
-      <c r="F24" s="28" t="n">
+      <c r="F24" s="25" t="n">
         <f aca="false">IF(C24=0,"",D24/C24)</f>
         <v>0.758635208840407</v>
       </c>
-      <c r="G24" s="28" t="n">
+      <c r="G24" s="25" t="n">
         <f aca="false">IF(C24=0,"",E24/C24)</f>
         <v>0.00656279425089275</v>
       </c>
-      <c r="H24" s="29"/>
-      <c r="I24" s="30"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="26" t="s">
+      <c r="H24" s="26"/>
+      <c r="I24" s="27"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="27" t="n">
+      <c r="C25" s="14" t="n">
         <v>472743</v>
       </c>
-      <c r="D25" s="27" t="n">
+      <c r="D25" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="28" t="n">
+      <c r="F25" s="25" t="n">
         <f aca="false">IF(C25=0,"",D25/C25)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="28" t="n">
+      <c r="G25" s="25" t="n">
         <f aca="false">IF(C25=0,"",E25/C25)</f>
         <v>0</v>
       </c>
-      <c r="H25" s="29"/>
-      <c r="I25" s="30"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="26" t="s">
+      <c r="H25" s="26"/>
+      <c r="I25" s="27"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C26" s="14" t="n">
         <v>407052</v>
       </c>
-      <c r="D26" s="27" t="n">
+      <c r="D26" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="28" t="n">
+      <c r="F26" s="25" t="n">
         <f aca="false">IF(C26=0,"",D26/C26)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="28" t="n">
+      <c r="G26" s="25" t="n">
         <f aca="false">IF(C26=0,"",E26/C26)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="29"/>
-      <c r="I26" s="30"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="26" t="s">
+      <c r="H26" s="26"/>
+      <c r="I26" s="27"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C27" s="27" t="n">
+      <c r="C27" s="14" t="n">
         <v>323878</v>
       </c>
-      <c r="D27" s="27" t="n">
+      <c r="D27" s="14" t="n">
         <v>323878</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="28" t="n">
+      <c r="F27" s="25" t="n">
         <f aca="false">IF(C27=0,"",D27/C27)</f>
         <v>1</v>
       </c>
-      <c r="G27" s="28" t="n">
+      <c r="G27" s="25" t="n">
         <f aca="false">IF(C27=0,"",E27/C27)</f>
         <v>0</v>
       </c>
-      <c r="H27" s="29"/>
-      <c r="I27" s="30"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="26" t="s">
+      <c r="H27" s="26"/>
+      <c r="I27" s="27"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C28" s="27" t="n">
+      <c r="C28" s="14" t="n">
         <v>298250</v>
       </c>
-      <c r="D28" s="27" t="n">
+      <c r="D28" s="14" t="n">
         <v>298250</v>
       </c>
-      <c r="E28" s="27" t="n">
+      <c r="E28" s="14" t="n">
         <v>276</v>
       </c>
-      <c r="F28" s="28" t="n">
+      <c r="F28" s="25" t="n">
         <f aca="false">IF(C28=0,"",D28/C28)</f>
         <v>1</v>
       </c>
-      <c r="G28" s="28" t="n">
+      <c r="G28" s="25" t="n">
         <f aca="false">IF(C28=0,"",E28/C28)</f>
         <v>0.000925398155909472</v>
       </c>
-      <c r="H28" s="29"/>
-      <c r="I28" s="30"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="26" t="s">
+      <c r="H28" s="26"/>
+      <c r="I28" s="27"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C29" s="27" t="n">
+      <c r="C29" s="14" t="n">
         <v>292081</v>
       </c>
-      <c r="D29" s="27" t="n">
+      <c r="D29" s="14" t="n">
         <v>292081</v>
       </c>
-      <c r="E29" s="27" t="n">
+      <c r="E29" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="28" t="n">
+      <c r="F29" s="25" t="n">
         <f aca="false">IF(C29=0,"",D29/C29)</f>
         <v>1</v>
       </c>
-      <c r="G29" s="28" t="n">
+      <c r="G29" s="25" t="n">
         <f aca="false">IF(C29=0,"",E29/C29)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="29"/>
-      <c r="I29" s="30"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="26" t="s">
+      <c r="H29" s="26"/>
+      <c r="I29" s="27"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="27" t="n">
+      <c r="C30" s="14" t="n">
         <v>166208</v>
       </c>
-      <c r="D30" s="27" t="n">
+      <c r="D30" s="14" t="n">
         <v>166208</v>
       </c>
-      <c r="E30" s="27" t="n">
+      <c r="E30" s="14" t="n">
         <v>628</v>
       </c>
-      <c r="F30" s="28" t="n">
+      <c r="F30" s="25" t="n">
         <f aca="false">IF(C30=0,"",D30/C30)</f>
         <v>1</v>
       </c>
-      <c r="G30" s="28" t="n">
+      <c r="G30" s="25" t="n">
         <f aca="false">IF(C30=0,"",E30/C30)</f>
         <v>0.00377839815171352</v>
       </c>
-      <c r="H30" s="29"/>
-      <c r="I30" s="30"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="26" t="s">
+      <c r="H30" s="26"/>
+      <c r="I30" s="27"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C31" s="27" t="n">
+      <c r="C31" s="14" t="n">
         <v>148542</v>
       </c>
-      <c r="D31" s="27" t="n">
+      <c r="D31" s="14" t="n">
         <v>148542</v>
       </c>
-      <c r="E31" s="27" t="n">
+      <c r="E31" s="14" t="n">
         <v>11170</v>
       </c>
-      <c r="F31" s="28" t="n">
+      <c r="F31" s="25" t="n">
         <f aca="false">IF(C31=0,"",D31/C31)</f>
         <v>1</v>
       </c>
-      <c r="G31" s="28" t="n">
+      <c r="G31" s="25" t="n">
         <f aca="false">IF(C31=0,"",E31/C31)</f>
         <v>0.0751975872143905</v>
       </c>
-      <c r="H31" s="29"/>
-      <c r="I31" s="30"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="26" t="s">
+      <c r="H31" s="26"/>
+      <c r="I31" s="27"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C32" s="27" t="n">
+      <c r="C32" s="14" t="n">
         <v>84835</v>
       </c>
-      <c r="D32" s="27" t="n">
+      <c r="D32" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="27" t="n">
+      <c r="E32" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="28" t="n">
+      <c r="F32" s="25" t="n">
         <f aca="false">IF(C32=0,"",D32/C32)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="28" t="n">
+      <c r="G32" s="25" t="n">
         <f aca="false">IF(C32=0,"",E32/C32)</f>
         <v>0</v>
       </c>
-      <c r="H32" s="29"/>
-      <c r="I32" s="30"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="26" t="s">
+      <c r="H32" s="26"/>
+      <c r="I32" s="27"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="C33" s="27" t="n">
+      <c r="C33" s="14" t="n">
         <v>3521</v>
       </c>
-      <c r="D33" s="27" t="n">
+      <c r="D33" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="27" t="n">
+      <c r="E33" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="28" t="n">
+      <c r="F33" s="25" t="n">
         <f aca="false">IF(C33=0,"",D33/C33)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="28" t="n">
+      <c r="G33" s="25" t="n">
         <f aca="false">IF(C33=0,"",E33/C33)</f>
         <v>0</v>
       </c>
-      <c r="H33" s="29"/>
-      <c r="I33" s="30"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="32" t="s">
+      <c r="H33" s="26"/>
+      <c r="I33" s="27"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C34" s="33" t="n">
+      <c r="C34" s="29" t="n">
         <f aca="false">SUM(C6:C33)</f>
         <v>203388298</v>
       </c>
-      <c r="D34" s="33" t="n">
+      <c r="D34" s="29" t="n">
         <f aca="false">SUM(D6:D33)</f>
         <v>119016969</v>
       </c>
-      <c r="E34" s="33" t="n">
+      <c r="E34" s="29" t="n">
         <f aca="false">SUM(E6:E33)</f>
         <v>9951387</v>
       </c>
-      <c r="F34" s="28" t="n">
+      <c r="F34" s="25" t="n">
         <f aca="false">D34/C34</f>
         <v>0.585171173417263</v>
       </c>
-      <c r="G34" s="28" t="n">
+      <c r="G34" s="25" t="n">
         <f aca="false">E34/C34</f>
         <v>0.0489280214144867</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="32" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C35" s="27" t="n">
+      <c r="C35" s="14" t="n">
         <v>203388298</v>
       </c>
-      <c r="D35" s="27" t="n">
+      <c r="D35" s="14" t="n">
         <v>119016969</v>
       </c>
-      <c r="E35" s="27" t="n">
+      <c r="E35" s="14" t="n">
         <v>9951387</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="34" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="3" t="s">
         <v>127</v>
       </c>
     </row>
@@ -4206,106 +4405,106 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="30" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="30" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="32" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="32" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="32" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="32" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="32" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="32" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="32" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="32" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="32" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="32" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="32" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="32" t="s">
         <v>153</v>
       </c>
     </row>
@@ -4334,7 +4533,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="33" t="s">
         <v>154</v>
       </c>
     </row>
@@ -4356,7 +4555,7 @@
       <c r="B4" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="34" t="s">
         <v>158</v>
       </c>
     </row>
@@ -4367,7 +4566,7 @@
       <c r="B5" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="34" t="s">
         <v>161</v>
       </c>
     </row>
@@ -4378,7 +4577,7 @@
       <c r="B6" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="34" t="s">
         <v>164</v>
       </c>
     </row>
@@ -4389,7 +4588,7 @@
       <c r="B7" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="C7" s="39"/>
+      <c r="C7" s="34"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
@@ -4398,7 +4597,7 @@
       <c r="B8" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="34" t="s">
         <v>169</v>
       </c>
     </row>
@@ -4409,7 +4608,7 @@
       <c r="B9" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="34" t="s">
         <v>172</v>
       </c>
     </row>
@@ -4420,7 +4619,7 @@
       <c r="B10" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="34" t="s">
         <v>175</v>
       </c>
     </row>
@@ -4431,7 +4630,7 @@
       <c r="B11" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="C11" s="39"/>
+      <c r="C11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -4440,7 +4639,7 @@
       <c r="B12" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="34" t="s">
         <v>180</v>
       </c>
     </row>
@@ -4451,7 +4650,7 @@
       <c r="B13" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="C13" s="34" t="s">
         <v>183</v>
       </c>
     </row>
@@ -4462,7 +4661,7 @@
       <c r="B14" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="34" t="s">
         <v>186</v>
       </c>
     </row>
@@ -4473,7 +4672,7 @@
       <c r="B15" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="34" t="s">
         <v>189</v>
       </c>
     </row>
@@ -4484,7 +4683,7 @@
       <c r="B16" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C16" s="39" t="s">
+      <c r="C16" s="34" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4495,7 +4694,7 @@
       <c r="B17" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="34" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4506,7 +4705,7 @@
       <c r="B18" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="34" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4517,7 +4716,7 @@
       <c r="B19" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="C19" s="39" t="s">
+      <c r="C19" s="34" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4528,7 +4727,7 @@
       <c r="B20" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="C20" s="39" t="s">
+      <c r="C20" s="34" t="s">
         <v>204</v>
       </c>
     </row>
@@ -4539,7 +4738,7 @@
       <c r="B21" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="C21" s="39" t="s">
+      <c r="C21" s="34" t="s">
         <v>207</v>
       </c>
     </row>
@@ -4550,7 +4749,7 @@
       <c r="B22" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="C22" s="39" t="s">
+      <c r="C22" s="34" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4561,7 +4760,7 @@
       <c r="B23" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="C23" s="39"/>
+      <c r="C23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
@@ -4570,7 +4769,7 @@
       <c r="B24" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="C24" s="34" t="s">
         <v>215</v>
       </c>
     </row>
@@ -4581,7 +4780,7 @@
       <c r="B25" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="C25" s="39"/>
+      <c r="C25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
@@ -4590,7 +4789,7 @@
       <c r="B26" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="34" t="s">
         <v>220</v>
       </c>
     </row>
@@ -4601,7 +4800,7 @@
       <c r="B27" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="C27" s="39" t="s">
+      <c r="C27" s="34" t="s">
         <v>223</v>
       </c>
     </row>
@@ -4612,7 +4811,7 @@
       <c r="B28" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="34" t="s">
         <v>226</v>
       </c>
     </row>
@@ -4623,7 +4822,7 @@
       <c r="B29" s="15" t="s">
         <v>228</v>
       </c>
-      <c r="C29" s="39" t="s">
+      <c r="C29" s="34" t="s">
         <v>229</v>
       </c>
     </row>
@@ -4634,7 +4833,7 @@
       <c r="B30" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="C30" s="39" t="s">
+      <c r="C30" s="34" t="s">
         <v>232</v>
       </c>
     </row>
@@ -4645,7 +4844,7 @@
       <c r="B31" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="C31" s="39" t="s">
+      <c r="C31" s="34" t="s">
         <v>235</v>
       </c>
     </row>
@@ -4656,7 +4855,7 @@
       <c r="B32" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="C32" s="39" t="s">
+      <c r="C32" s="34" t="s">
         <v>238</v>
       </c>
     </row>
@@ -4667,7 +4866,7 @@
       <c r="B33" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="C33" s="39" t="s">
+      <c r="C33" s="34" t="s">
         <v>241</v>
       </c>
     </row>
@@ -4678,7 +4877,7 @@
       <c r="B34" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="C34" s="39" t="s">
+      <c r="C34" s="34" t="s">
         <v>244</v>
       </c>
     </row>
@@ -4689,7 +4888,7 @@
       <c r="B35" s="15" t="s">
         <v>246</v>
       </c>
-      <c r="C35" s="39" t="s">
+      <c r="C35" s="34" t="s">
         <v>247</v>
       </c>
     </row>
@@ -4700,7 +4899,7 @@
       <c r="B36" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="C36" s="39" t="s">
+      <c r="C36" s="34" t="s">
         <v>250</v>
       </c>
     </row>
@@ -4713,4 +4912,370 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B1:G41"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="35" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="37" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="38" t="s">
+        <v>254</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="39" t="s">
+        <v>256</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>7236</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="39" t="s">
+        <v>257</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>8839</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="39" t="s">
+        <v>258</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>9093</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="39" t="s">
+        <v>259</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>12118</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="39" t="s">
+        <v>260</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>14697</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="41" t="s">
+        <v>263</v>
+      </c>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="37" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="C18" s="40" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="39" t="s">
+        <v>267</v>
+      </c>
+      <c r="C20" s="40" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="39" t="s">
+        <v>269</v>
+      </c>
+      <c r="C22" s="40" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="37" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="38" t="s">
+        <v>272</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>273</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>274</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="39" t="s">
+        <v>276</v>
+      </c>
+      <c r="C26" s="39" t="s">
+        <v>277</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="E26" s="39" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="C27" s="39" t="s">
+        <v>281</v>
+      </c>
+      <c r="D27" s="39" t="s">
+        <v>282</v>
+      </c>
+      <c r="E27" s="39" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="39" t="s">
+        <v>284</v>
+      </c>
+      <c r="C28" s="39" t="s">
+        <v>285</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>286</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="39" t="s">
+        <v>288</v>
+      </c>
+      <c r="C29" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="D29" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="39" t="s">
+        <v>291</v>
+      </c>
+      <c r="C30" s="39" t="s">
+        <v>292</v>
+      </c>
+      <c r="D30" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="39" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="39" t="s">
+        <v>294</v>
+      </c>
+      <c r="C31" s="39" t="s">
+        <v>295</v>
+      </c>
+      <c r="D31" s="39" t="s">
+        <v>296</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="39" t="s">
+        <v>298</v>
+      </c>
+      <c r="C32" s="39" t="s">
+        <v>299</v>
+      </c>
+      <c r="D32" s="39" t="s">
+        <v>300</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="37" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="42" t="s">
+        <v>303</v>
+      </c>
+      <c r="C35" s="42"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="42"/>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="42" t="s">
+        <v>304</v>
+      </c>
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+    </row>
+    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="42" t="s">
+        <v>305</v>
+      </c>
+      <c r="C37" s="42"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="42" t="s">
+        <v>306</v>
+      </c>
+      <c r="C38" s="42"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="42"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+    </row>
+    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="42" t="s">
+        <v>307</v>
+      </c>
+      <c r="C39" s="42"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="43" t="s">
+        <v>308</v>
+      </c>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B2:G3"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B41:G41"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add UPERC FY27 tariff order disclosures: PMPM rates, opex disallowance, TBCB-vs-AMISP regulatory contrast
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Consumer_Metering_Status_Aug2026.xlsx
+++ b/Smart_Consumer_Metering_Status_Aug2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="341">
   <si>
     <t xml:space="preserve">Smart Consumer Metering Status as on 20-Aug-2026</t>
   </si>
@@ -951,6 +951,102 @@
   </si>
   <si>
     <t xml:space="preserve">Sources: Prayas (Energy Group) Apr-2025 (RDSS dashboard compilation); ThePrint 24-Oct-22; T&amp;D India 22-Sep-23 &amp; 15-Jun-26; Tehelka Jul-26; CareEdge Mar-2025; Genus Q4FY26 call transcript; Tata Power release.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5) Regulatory disclosure route — why there is no TBCB-style L1 data, and what the ARR route reveals (UPERC FY27 Tariff Order, uperc.org, 501 pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Transmission TBCB: bid under Sec 63 Electricity Act -&gt; mandatory tariff ADOPTION petition before CERC/SERC -&gt; public orders disclose L1 levelized tariff and bidder lists.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- AMISP: service procurement under MoP SBD (TOTEX, 93-month O&amp;M) — NOT a Sec 63 tariff -&gt; no adoption petition -&gt; L1/L2 never published. Disclosure happens only when the discom seeks recovery in its ARR (SBD clause 9(ix): AMISP service charge + lumpsum to be treated as opex in ARR filings).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the UPERC FY26-27 Tariff Order (UPPCL discoms) actually discloses:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EESL legacy PMPM (disclosed rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.101.421 /meter/month incl. GST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DVVNL, MVVNL, PVVNL, PuVVNL; KESCO Rs.85.95. 47.09 lakh EESL meters; Rs.138.08 cr paid FY24-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate first claimed by discoms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.114.57 /meter/month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revised down to Rs.101.421 after Commission's deficiency query</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY24-25 true-up claim vs actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.363.75 cr claimed vs Rs.138.08 cr actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission: 'excessive and unjustified'; RDSS AMISP expense not booked in FY24-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26-27 Smart Metering Opex claimed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.3,837.54 cr (consolidated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DVVNL 774.47 + MVVNL 1,008.94 + PVVNL 799.41 + PuVVNL 1,109.97 + KESCO 144.74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26-27 approved by UPERC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs. 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disallowed entirely: scheme is 'self-sustaining' — opex must be absorbed via billing/collection gains, not passed to consumers; door left open at true-up if savings data furnished</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MoP letter 16-Sep-2023 to all SERCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'no extra cost be passed on to consumers'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cites net GAIN of ~Rs.40/meter/month after AMISP opex (power purchase + billing savings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MoP advisory 28-Nov-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allow smart metering expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERCs advised to permit recovery for cost-reflective tariffs — the two directions now in tension; UPERC 'harmonised': allow only where demonstrated savings &gt;= expense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RDSS package-wise PMPM rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitted, not printed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discoms filed package-wise approved PMPM rates + Rs.900/meter lumpsum billing with the Commission (para 6.8.18) — in petition annexures, not the public order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consumer-charge case (suo motu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs.33.22 cr excess / 93,138 connections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep-25 to Jan-26: charged above the 2019 Cost Data Book rate (Rs.6,016 single-phase); 100% credit ordered; press reports ~Rs.200 cr refunds to 5+ lakh consumers ordered Mar/Apr-26; hearings ongoing Aug-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Investor takeaway: the PMPM won in bidding is contractually payable by discoms regardless of ARR treatment (DDF-secured), but UP shows recovery from consumers is contested — a discom-credit-risk overhang on AMISP annuities, not an AMISP revenue risk per se. Source: UPERC ARR &amp; Tariff Order FY2026-27 (www.uperc.org/App_File/UPPCLTariffOrder-pdf72202630517PM.pdf); Saur Energy Mar-26 &amp; Aug-26.</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1237,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1282,20 +1378,8 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1316,6 +1400,14 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1528,8 +1620,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="88362268"/>
-        <c:axId val="51747353"/>
+        <c:axId val="63955391"/>
+        <c:axId val="31888231"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1642,11 +1734,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="88362268"/>
-        <c:axId val="51747353"/>
+        <c:axId val="63955391"/>
+        <c:axId val="31888231"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="88362268"/>
+        <c:axId val="63955391"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1678,7 +1770,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51747353"/>
+        <c:crossAx val="31888231"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1686,7 +1778,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51747353"/>
+        <c:axId val="31888231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1728,7 +1820,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88362268"/>
+        <c:crossAx val="63955391"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2096,11 +2188,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="6985815"/>
-        <c:axId val="79293854"/>
+        <c:axId val="81938988"/>
+        <c:axId val="96710758"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6985815"/>
+        <c:axId val="81938988"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2132,7 +2224,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79293854"/>
+        <c:crossAx val="96710758"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2140,7 +2232,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79293854"/>
+        <c:axId val="96710758"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2182,7 +2274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6985815"/>
+        <c:crossAx val="81938988"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2526,9 +2618,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>125280</xdr:colOff>
+      <xdr:colOff>124920</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>16920</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2537,7 +2629,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="566640"/>
-        <a:ext cx="4678200" cy="2698200"/>
+        <a:ext cx="4677840" cy="2697840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2556,9 +2648,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>47520</xdr:colOff>
+      <xdr:colOff>47160</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>6120</xdr:rowOff>
+      <xdr:rowOff>5760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2567,7 +2659,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="3614040"/>
-        <a:ext cx="6118200" cy="2878560"/>
+        <a:ext cx="6117840" cy="2878200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2586,9 +2678,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>164160</xdr:colOff>
+      <xdr:colOff>163800</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>16920</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2597,7 +2689,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14538240" y="7424640"/>
-        <a:ext cx="3958200" cy="2698200"/>
+        <a:ext cx="3957840" cy="2697840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4919,348 +5011,498 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:G41"/>
+  <dimension ref="B1:G60"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="35" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="23" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="35" t="s">
         <v>252</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="37" t="s">
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="38" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="5" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="39" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="36" t="s">
         <v>256</v>
       </c>
-      <c r="C7" s="40" t="n">
+      <c r="C7" s="37" t="n">
         <v>7236</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="39" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="C8" s="40" t="n">
+      <c r="C8" s="37" t="n">
         <v>8839</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="39" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="36" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="40" t="n">
+      <c r="C9" s="37" t="n">
         <v>9093</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="39" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="36" t="s">
         <v>259</v>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="37" t="n">
         <v>12118</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="39" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="36" t="s">
         <v>260</v>
       </c>
-      <c r="C11" s="40" t="n">
+      <c r="C11" s="37" t="n">
         <v>14697</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="39" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="C12" s="40" t="s">
+      <c r="C12" s="37" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="37" t="s">
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="38" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="5" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="39" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="C18" s="40" t="n">
+      <c r="C18" s="37" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="39" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="40" t="n">
+      <c r="C19" s="37" t="n">
         <v>79</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="39" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="36" t="s">
         <v>267</v>
       </c>
-      <c r="C20" s="40" t="n">
+      <c r="C20" s="37" t="n">
         <v>146</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="39" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="36" t="s">
         <v>268</v>
       </c>
-      <c r="C21" s="40" t="n">
+      <c r="C21" s="37" t="n">
         <v>167</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="39" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="36" t="s">
         <v>269</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="37" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="37" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="38" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="C25" s="38" t="s">
+      <c r="C25" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="E25" s="38" t="s">
+      <c r="E25" s="5" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="36" t="s">
         <v>276</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="36" t="s">
         <v>277</v>
       </c>
-      <c r="D26" s="39" t="s">
+      <c r="D26" s="36" t="s">
         <v>278</v>
       </c>
-      <c r="E26" s="39" t="s">
+      <c r="E26" s="36" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="39" t="s">
+      <c r="B27" s="36" t="s">
         <v>280</v>
       </c>
-      <c r="C27" s="39" t="s">
+      <c r="C27" s="36" t="s">
         <v>281</v>
       </c>
-      <c r="D27" s="39" t="s">
+      <c r="D27" s="36" t="s">
         <v>282</v>
       </c>
-      <c r="E27" s="39" t="s">
+      <c r="E27" s="36" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="39" t="s">
+      <c r="B28" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="D28" s="39" t="s">
+      <c r="D28" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="E28" s="39" t="s">
+      <c r="E28" s="36" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="39" t="s">
+      <c r="B29" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="C29" s="39" t="s">
+      <c r="C29" s="36" t="s">
         <v>289</v>
       </c>
-      <c r="D29" s="39" t="s">
+      <c r="D29" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="E29" s="36" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="36" t="s">
         <v>291</v>
       </c>
-      <c r="C30" s="39" t="s">
+      <c r="C30" s="36" t="s">
         <v>292</v>
       </c>
-      <c r="D30" s="39" t="s">
+      <c r="D30" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="E30" s="39" t="s">
+      <c r="E30" s="36" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="39" t="s">
+      <c r="B31" s="36" t="s">
         <v>294</v>
       </c>
-      <c r="C31" s="39" t="s">
+      <c r="C31" s="36" t="s">
         <v>295</v>
       </c>
-      <c r="D31" s="39" t="s">
+      <c r="D31" s="36" t="s">
         <v>296</v>
       </c>
-      <c r="E31" s="39" t="s">
+      <c r="E31" s="36" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="39" t="s">
+      <c r="B32" s="36" t="s">
         <v>298</v>
       </c>
-      <c r="C32" s="39" t="s">
+      <c r="C32" s="36" t="s">
         <v>299</v>
       </c>
-      <c r="D32" s="39" t="s">
+      <c r="D32" s="36" t="s">
         <v>300</v>
       </c>
-      <c r="E32" s="39" t="s">
+      <c r="E32" s="36" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="37" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="42" t="s">
+      <c r="B35" s="39" t="s">
         <v>303</v>
       </c>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="42" t="s">
+      <c r="B36" s="39" t="s">
         <v>304</v>
       </c>
-      <c r="C36" s="42"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
     </row>
     <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="42" t="s">
+      <c r="B37" s="39" t="s">
         <v>305</v>
       </c>
-      <c r="C37" s="42"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="42"/>
-      <c r="F37" s="42"/>
-      <c r="G37" s="42"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
     </row>
     <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="42" t="s">
+      <c r="B38" s="39" t="s">
         <v>306</v>
       </c>
-      <c r="C38" s="42"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="42"/>
-      <c r="F38" s="42"/>
-      <c r="G38" s="42"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
     </row>
     <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="39" t="s">
         <v>307</v>
       </c>
-      <c r="C39" s="42"/>
-      <c r="D39" s="42"/>
-      <c r="E39" s="42"/>
-      <c r="F39" s="42"/>
-      <c r="G39" s="42"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="43" t="s">
+      <c r="B41" s="40" t="s">
         <v>308</v>
       </c>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
+      <c r="G41" s="40"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="41" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="39" t="s">
+        <v>310</v>
+      </c>
+      <c r="C45" s="39"/>
+      <c r="D45" s="39"/>
+      <c r="E45" s="39"/>
+      <c r="F45" s="39"/>
+      <c r="G45" s="39"/>
+    </row>
+    <row r="46" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="39" t="s">
+        <v>311</v>
+      </c>
+      <c r="C46" s="39"/>
+      <c r="D46" s="39"/>
+      <c r="E46" s="39"/>
+      <c r="F46" s="39"/>
+      <c r="G46" s="39"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="41" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="D49" s="42" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="36" t="s">
+        <v>313</v>
+      </c>
+      <c r="C50" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="D50" s="34" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="36" t="s">
+        <v>316</v>
+      </c>
+      <c r="C51" s="37" t="s">
+        <v>317</v>
+      </c>
+      <c r="D51" s="34" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B52" s="36" t="s">
+        <v>319</v>
+      </c>
+      <c r="C52" s="37" t="s">
+        <v>320</v>
+      </c>
+      <c r="D52" s="34" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="36" t="s">
+        <v>322</v>
+      </c>
+      <c r="C53" s="37" t="s">
+        <v>323</v>
+      </c>
+      <c r="D53" s="34" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="36" t="s">
+        <v>325</v>
+      </c>
+      <c r="C54" s="37" t="s">
+        <v>326</v>
+      </c>
+      <c r="D54" s="34" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="36" t="s">
+        <v>328</v>
+      </c>
+      <c r="C55" s="37" t="s">
+        <v>329</v>
+      </c>
+      <c r="D55" s="34" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="36" t="s">
+        <v>331</v>
+      </c>
+      <c r="C56" s="37" t="s">
+        <v>332</v>
+      </c>
+      <c r="D56" s="34" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B57" s="36" t="s">
+        <v>334</v>
+      </c>
+      <c r="C57" s="37" t="s">
+        <v>335</v>
+      </c>
+      <c r="D57" s="34" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="36" t="s">
+        <v>337</v>
+      </c>
+      <c r="C58" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="D58" s="34" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B60" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="C60" s="39"/>
+      <c r="D60" s="39"/>
+      <c r="E60" s="39"/>
+      <c r="F60" s="39"/>
+      <c r="G60" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
     <mergeCell ref="B2:G3"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B35:G35"/>
@@ -5269,6 +5511,9 @@
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="B39:G39"/>
     <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B60:G60"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>